<commit_message>
uploaded updated courts list file
</commit_message>
<xml_diff>
--- a/docassemble/RFApackage/data/sources/courts_list.xlsx
+++ b/docassemble/RFApackage/data/sources/courts_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miabonardi/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vtlegalaid-my.sharepoint.com/personal/ksurette_lawlinevt_org/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE7CE2C-E5E2-C541-A927-DC623C8D6ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{CF2E742D-44F9-4086-A5A6-A69C6F7ADFC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36400547-8786-4530-91D1-7F050F48CF02}"/>
   <bookViews>
-    <workbookView xWindow="6900" yWindow="1120" windowWidth="29040" windowHeight="15840" xr2:uid="{F13D4BD2-1651-4B43-8F6C-36F85B10F0AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F13D4BD2-1651-4B43-8F6C-36F85B10F0AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="97">
   <si>
     <t>name</t>
   </si>
@@ -212,42 +212,6 @@
     <t>802-295-8865</t>
   </si>
   <si>
-    <t>JUD.AddisonUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.BenningtonUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.CaledoniaEssexUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.ChittendenUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.FranklinGrandIsleunit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.LamoilleUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.OrangeUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.OrleansUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.RutlandUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.WashingtonUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.WindhamUnit@vermont.gov</t>
-  </si>
-  <si>
-    <t>JUD.WindsorUnit@vermont.gov</t>
-  </si>
-  <si>
     <t>PO Box 75, Guildhall, VT 05905</t>
   </si>
   <si>
@@ -321,6 +285,48 @@
   </si>
   <si>
     <t>arbitrary_attribute</t>
+  </si>
+  <si>
+    <t>division_abbr</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>BenningtonUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>CaledoniaEssexUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>ChittendenUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>FranklinGrandIsleunit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>LamoilleUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>OrangeUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>OrleansUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>RutlandUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>WashingtonUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>WindhamUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>WindsorUnit@vtcourts.gov</t>
+  </si>
+  <si>
+    <t>AddisonUnit@vtcourts.gov</t>
   </si>
 </sst>
 </file>
@@ -330,7 +336,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="00000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -342,6 +348,14 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -394,10 +408,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -409,8 +424,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -427,9 +444,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -467,7 +484,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -573,7 +590,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -715,7 +732,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -723,28 +740,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3A491E8-E2DE-9A4E-A3B9-C224836C99FE}">
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:T15"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.83203125" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="7" max="7" width="4.1640625" customWidth="1"/>
-    <col min="8" max="8" width="36.1640625" customWidth="1"/>
-    <col min="9" max="9" width="31.6640625" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="29.1640625" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-    <col min="17" max="17" width="17.6640625" customWidth="1"/>
-    <col min="18" max="18" width="16.83203125" customWidth="1"/>
-    <col min="19" max="19" width="19.6640625" customWidth="1"/>
+    <col min="1" max="1" width="23.875" customWidth="1"/>
+    <col min="2" max="2" width="7.125" customWidth="1"/>
+    <col min="4" max="5" width="15" customWidth="1"/>
+    <col min="8" max="8" width="4.125" customWidth="1"/>
+    <col min="9" max="9" width="36.125" customWidth="1"/>
+    <col min="10" max="10" width="31.625" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="14.875" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="15" max="15" width="15.375" customWidth="1"/>
+    <col min="16" max="16" width="29.125" customWidth="1"/>
+    <col min="17" max="17" width="20.875" customWidth="1"/>
+    <col min="18" max="18" width="17.625" customWidth="1"/>
+    <col min="19" max="19" width="16.875" customWidth="1"/>
+    <col min="20" max="20" width="19.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -758,52 +775,55 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
-        <v>94</v>
+      <c r="T1" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -813,38 +833,41 @@
       <c r="D2" t="s">
         <v>18</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" t="s">
         <v>44</v>
       </c>
-      <c r="H2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="I2" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>21</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="5">
+      <c r="N2" s="5">
         <v>5753</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>20</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>44.013869999999997</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>-73.162989999999994</v>
       </c>
-      <c r="R2" t="s">
-        <v>92</v>
+      <c r="S2" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -854,38 +877,41 @@
       <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" t="s">
         <v>45</v>
       </c>
-      <c r="H3" t="s">
-        <v>59</v>
-      </c>
-      <c r="I3" t="s">
-        <v>77</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="I3" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="J3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" t="s">
         <v>24</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="6">
+      <c r="N3" s="6">
         <v>5201</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>24</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>42.888089999999998</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>-73.198170000000005</v>
       </c>
-      <c r="R3" t="s">
-        <v>92</v>
+      <c r="S3" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -895,41 +921,44 @@
       <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" t="s">
         <v>46</v>
       </c>
-      <c r="H4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" t="s">
-        <v>81</v>
+      <c r="I4" s="7" t="s">
+        <v>86</v>
       </c>
       <c r="J4" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="K4" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="L4" t="s">
+        <v>61</v>
+      </c>
+      <c r="M4" t="s">
         <v>22</v>
       </c>
-      <c r="M4" s="6">
+      <c r="N4" s="6">
         <v>5819</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>33</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>44.417960000000001</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>-72.020300000000006</v>
       </c>
-      <c r="R4" t="s">
-        <v>92</v>
+      <c r="S4" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -939,41 +968,44 @@
       <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" t="s">
         <v>47</v>
       </c>
-      <c r="H5" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" t="s">
-        <v>82</v>
+      <c r="I5" s="7" t="s">
+        <v>87</v>
       </c>
       <c r="J5" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="K5" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="L5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="6">
+      <c r="N5" s="6">
         <v>5401</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>34</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>44.47945</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>-73.217330000000004</v>
       </c>
-      <c r="R5" t="s">
-        <v>92</v>
+      <c r="S5" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -983,35 +1015,38 @@
       <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E6" t="s">
+        <v>84</v>
+      </c>
+      <c r="G6" t="s">
         <v>48</v>
       </c>
-      <c r="H6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I6" t="s">
-        <v>93</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="I6" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="J6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" t="s">
         <v>25</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="6">
+      <c r="N6" s="6">
         <v>5905</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>35</v>
       </c>
-      <c r="R6" t="s">
-        <v>92</v>
-      </c>
       <c r="S6" t="s">
-        <v>70</v>
+        <v>80</v>
+      </c>
+      <c r="T6" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1021,32 +1056,35 @@
       <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" t="s">
+      <c r="E7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" t="s">
         <v>49</v>
       </c>
-      <c r="H7" t="s">
-        <v>62</v>
-      </c>
-      <c r="I7" t="s">
-        <v>83</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="I7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" t="s">
+        <v>71</v>
+      </c>
+      <c r="L7" t="s">
         <v>26</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="6">
+      <c r="N7" s="6">
         <v>5478</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>36</v>
       </c>
-      <c r="R7" t="s">
-        <v>92</v>
+      <c r="S7" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1056,35 +1094,38 @@
       <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="F8" t="s">
+      <c r="E8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" t="s">
         <v>50</v>
       </c>
-      <c r="H8" t="s">
-        <v>62</v>
-      </c>
-      <c r="I8" t="s">
-        <v>84</v>
-      </c>
-      <c r="K8" t="s">
+      <c r="I8" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J8" t="s">
+        <v>72</v>
+      </c>
+      <c r="L8" t="s">
         <v>27</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>22</v>
       </c>
-      <c r="M8" s="6">
+      <c r="N8" s="6">
         <v>5474</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>37</v>
       </c>
-      <c r="R8" t="s">
-        <v>92</v>
-      </c>
       <c r="S8" t="s">
-        <v>71</v>
+        <v>80</v>
+      </c>
+      <c r="T8" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1094,35 +1135,38 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="F9" t="s">
+      <c r="E9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" t="s">
         <v>51</v>
       </c>
-      <c r="H9" t="s">
-        <v>63</v>
-      </c>
-      <c r="I9" t="s">
-        <v>85</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="I9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="J9" t="s">
+        <v>73</v>
+      </c>
+      <c r="L9" t="s">
         <v>28</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="6">
+      <c r="N9" s="6">
         <v>5655</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" t="s">
-        <v>92</v>
-      </c>
       <c r="S9" t="s">
-        <v>72</v>
+        <v>80</v>
+      </c>
+      <c r="T9" t="s">
+        <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1132,32 +1176,35 @@
       <c r="D10" t="s">
         <v>18</v>
       </c>
-      <c r="F10" t="s">
+      <c r="E10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" t="s">
         <v>52</v>
       </c>
-      <c r="H10" t="s">
-        <v>64</v>
-      </c>
-      <c r="I10" t="s">
-        <v>86</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="I10" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J10" t="s">
+        <v>74</v>
+      </c>
+      <c r="L10" t="s">
         <v>29</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>22</v>
       </c>
-      <c r="M10" s="6">
+      <c r="N10" s="6">
         <v>5038</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>39</v>
       </c>
-      <c r="R10" t="s">
-        <v>92</v>
+      <c r="S10" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1167,35 +1214,38 @@
       <c r="D11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" t="s">
+      <c r="E11" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" t="s">
         <v>53</v>
       </c>
-      <c r="H11" t="s">
-        <v>65</v>
-      </c>
-      <c r="I11" t="s">
-        <v>87</v>
+      <c r="I11" s="7" t="s">
+        <v>91</v>
       </c>
       <c r="J11" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K11" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
+        <v>63</v>
+      </c>
+      <c r="M11" t="s">
         <v>22</v>
       </c>
-      <c r="M11" s="6">
+      <c r="N11" s="6">
         <v>5855</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>40</v>
       </c>
-      <c r="R11" t="s">
-        <v>92</v>
+      <c r="S11" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1205,32 +1255,35 @@
       <c r="D12" t="s">
         <v>18</v>
       </c>
-      <c r="F12" t="s">
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" t="s">
         <v>54</v>
       </c>
-      <c r="H12" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" t="s">
-        <v>88</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="I12" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" t="s">
+        <v>76</v>
+      </c>
+      <c r="L12" t="s">
         <v>30</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>22</v>
       </c>
-      <c r="M12" s="6">
+      <c r="N12" s="6">
         <v>5701</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>30</v>
       </c>
-      <c r="R12" t="s">
-        <v>92</v>
+      <c r="S12" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1240,35 +1293,38 @@
       <c r="D13" t="s">
         <v>18</v>
       </c>
-      <c r="F13" t="s">
+      <c r="E13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G13" t="s">
         <v>55</v>
       </c>
-      <c r="H13" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" t="s">
-        <v>89</v>
+      <c r="I13" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="J13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K13" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13" t="s">
         <v>31</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>22</v>
       </c>
-      <c r="M13" s="6">
+      <c r="N13" s="6">
         <v>5641</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>41</v>
       </c>
-      <c r="R13" t="s">
-        <v>92</v>
+      <c r="S13" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1278,35 +1334,38 @@
       <c r="D14" t="s">
         <v>18</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" t="s">
         <v>56</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" t="s">
+        <v>78</v>
+      </c>
+      <c r="K14" t="s">
         <v>68</v>
       </c>
-      <c r="I14" t="s">
-        <v>90</v>
-      </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
+        <v>64</v>
+      </c>
+      <c r="M14" t="s">
+        <v>22</v>
+      </c>
+      <c r="N14" s="6">
+        <v>5301</v>
+      </c>
+      <c r="O14" t="s">
+        <v>42</v>
+      </c>
+      <c r="S14" t="s">
         <v>80</v>
       </c>
-      <c r="K14" t="s">
-        <v>76</v>
-      </c>
-      <c r="L14" t="s">
-        <v>22</v>
-      </c>
-      <c r="M14" s="6">
-        <v>5301</v>
-      </c>
-      <c r="N14" t="s">
-        <v>42</v>
-      </c>
-      <c r="R14" t="s">
-        <v>92</v>
-      </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1316,33 +1375,52 @@
       <c r="D15" t="s">
         <v>18</v>
       </c>
-      <c r="F15" t="s">
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
         <v>57</v>
       </c>
-      <c r="H15" t="s">
-        <v>69</v>
-      </c>
-      <c r="I15" t="s">
-        <v>91</v>
-      </c>
-      <c r="K15" t="s">
+      <c r="I15" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15" t="s">
+        <v>79</v>
+      </c>
+      <c r="L15" t="s">
         <v>32</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>22</v>
       </c>
-      <c r="M15" s="6">
+      <c r="N15" s="6">
         <v>5001</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>43</v>
       </c>
-      <c r="R15" t="s">
-        <v>92</v>
+      <c r="S15" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" display="AddisonUnit@vermont.gov" xr:uid="{CE067579-4D2A-4FB7-BC20-71CF63E84A64}"/>
+    <hyperlink ref="I3" r:id="rId2" display="BenningtonUnit@vermont.gov" xr:uid="{FB72F267-E788-4851-A3D1-CA77ACFF585C}"/>
+    <hyperlink ref="I4" r:id="rId3" display="CaledoniaEssexUnit@vermont.gov" xr:uid="{1A175C18-6B0E-45DA-900D-8291E2C78C99}"/>
+    <hyperlink ref="I5" r:id="rId4" display="ChittendenUnit@vermont.gov" xr:uid="{9FF34C42-4441-46C0-BE1D-9155E2E8825B}"/>
+    <hyperlink ref="I6" r:id="rId5" display="CaledoniaEssexUnit@vermont.gov" xr:uid="{760AAC80-1B97-436E-AEB1-09E75778AC9D}"/>
+    <hyperlink ref="I7" r:id="rId6" display="FranklinGrandIsleunit@vermont.gov" xr:uid="{8F842D91-7453-45BA-A54E-CBCE4FE0577D}"/>
+    <hyperlink ref="I8" r:id="rId7" display="FranklinGrandIsleunit@vermont.gov" xr:uid="{7871886E-3C12-4CEC-B5B2-18622AD5509B}"/>
+    <hyperlink ref="I9" r:id="rId8" display="LamoilleUnit@vermont.gov" xr:uid="{69019928-95E2-41A0-9CD5-BDA65F0890D7}"/>
+    <hyperlink ref="I10" r:id="rId9" display="OrangeUnit@vermont.gov" xr:uid="{E536316C-27C7-4716-B9B2-FF9CE5C9D428}"/>
+    <hyperlink ref="I11" r:id="rId10" display="OrleansUnit@vermont.gov" xr:uid="{2F4F8B7F-2002-495A-A50F-5BC3EA27B661}"/>
+    <hyperlink ref="I12" r:id="rId11" display="RutlandUnit@vermont.gov" xr:uid="{E84206E9-32FD-488A-9404-A74109553EE1}"/>
+    <hyperlink ref="I13" r:id="rId12" display="WashingtonUnit@vermont.gov" xr:uid="{62688A28-3730-46D9-8F5B-6CB580AB3A11}"/>
+    <hyperlink ref="I14" r:id="rId13" display="WindhamUnit@vermont.gov" xr:uid="{AE616A9A-A9CF-473C-AA71-EF580C860226}"/>
+    <hyperlink ref="I15" r:id="rId14" display="WindsorUnit@vermont.gov" xr:uid="{79E27C0A-1083-4C5E-B394-01C1BC9FC0CD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>